<commit_message>
Fix: desactivar suavizado de líneas y usar gráfico de barras para índices de capacidad (P2)
</commit_message>
<xml_diff>
--- a/excel/solucion.xlsx
+++ b/excel/solucion.xlsx
@@ -219,6 +219,7 @@
               <f>'P1 Carta np'!$I$4:$I$23</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="1"/>
@@ -251,6 +252,7 @@
               <f>'P1 Carta np'!$J$4:$J$23</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="2"/>
@@ -283,6 +285,7 @@
               <f>'P1 Carta np'!$K$4:$K$23</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="3"/>
@@ -315,6 +318,7 @@
               <f>'P1 Carta np'!$L$4:$L$23</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -400,8 +404,9 @@
       </tx>
     </title>
     <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -415,14 +420,6 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
           <cat>
             <numRef>
               <f>'P2 Capacidad'!$A$12:$A$16</f>
@@ -434,9 +431,10 @@
             </numRef>
           </val>
         </ser>
+        <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
-      </lineChart>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -521,6 +519,7 @@
               <f>'P3 Carta X-R'!$M$4:$M$18</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="1"/>
@@ -553,6 +552,7 @@
               <f>'P3 Carta X-R'!$N$4:$N$18</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="2"/>
@@ -585,6 +585,7 @@
               <f>'P3 Carta X-R'!$O$4:$O$18</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="3"/>
@@ -617,6 +618,7 @@
               <f>'P3 Carta X-R'!$P$4:$P$18</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>

</xml_diff>

<commit_message>
Mejorar estilo visual de gráficas: colores UCL/CL/LCL diferenciados, marcadores, etiquetas de dato
</commit_message>
<xml_diff>
--- a/excel/solucion.xlsx
+++ b/excel/solucion.xlsx
@@ -197,13 +197,20 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:srgbClr val="2E5FA3"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="6"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E5FA3"/>
+              </a:solidFill>
               <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -230,8 +237,11 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
+            <a:ln w="15875">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
             </a:ln>
           </spPr>
           <marker>
@@ -263,7 +273,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln w="15875">
+              <a:solidFill>
+                <a:srgbClr val="1F7A4C"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -296,8 +309,11 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
+            <a:ln w="15875">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
             </a:ln>
           </spPr>
           <marker>
@@ -355,7 +371,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>
@@ -407,6 +422,7 @@
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="1"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -431,6 +447,9 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -452,15 +471,11 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -497,13 +512,20 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:srgbClr val="2E5FA3"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="6"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E5FA3"/>
+              </a:solidFill>
               <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -530,8 +552,11 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
+            <a:ln w="15875">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
             </a:ln>
           </spPr>
           <marker>
@@ -563,7 +588,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln w="15875">
+              <a:solidFill>
+                <a:srgbClr val="1F7A4C"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -596,8 +624,11 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
+            <a:ln w="15875">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
             </a:ln>
           </spPr>
           <marker>
@@ -655,7 +686,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>

</xml_diff>